<commit_message>
ARIA v2 final - renamed to aria.py
</commit_message>
<xml_diff>
--- a/SAT_Flight_Data.xlsx
+++ b/SAT_Flight_Data.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DeBoSSD/HAX/flight-chatbot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8025064C-ACE3-0C44-A64B-7CA0D5266536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9ECE110-30D7-4946-9FA9-C233EE887EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{4893EB22-DEF4-AD42-8CD7-323757C4E1C6}"/>
   </bookViews>
   <sheets>
-    <sheet name="arrivals" sheetId="1" r:id="rId1"/>
-    <sheet name="departures" sheetId="2" r:id="rId2"/>
+    <sheet name="Departures" sheetId="1" r:id="rId1"/>
+    <sheet name="Arrivals" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>

</xml_diff>